<commit_message>
Set BDTPTUMCF to 0 for hydrogen CT
</commit_message>
<xml_diff>
--- a/InputData/elec/BDTPTUMCF/Boolean Does This Plant Type Use Maximum Capacity Factor.xlsx
+++ b/InputData/elec/BDTPTUMCF/Boolean Does This Plant Type Use Maximum Capacity Factor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\BDTPTUMCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97DCE9AD-342C-4F1D-9344-9510E0382F11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F782727-4A9D-4E77-9E54-B70F49E4C0AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2370" yWindow="1695" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="12" r:id="rId1"/>
@@ -365,6 +365,9 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Header Descriptions"/>
       <sheetName val="2019 NQC List"/>
@@ -386,6 +389,9 @@
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Information"/>
       <sheetName val="Request Type 1-2"/>
@@ -1047,7 +1053,7 @@
         <v>31</v>
       </c>
       <c r="B24" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>